<commit_message>
Auto upload LP files
</commit_message>
<xml_diff>
--- a/lp_list.xlsx
+++ b/lp_list.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C420"/>
+  <dimension ref="A1:C421"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6724,6 +6724,21 @@
         </is>
       </c>
     </row>
+    <row r="421">
+      <c r="A421" t="n">
+        <v>496</v>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>Milli Vanili (밀리 바닐리)</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>Baby Don't Forget My Number</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>